<commit_message>
Actualización de habilidades, excels e imágenes
</commit_message>
<xml_diff>
--- a/Mercado Viejo (hay que cambiarlo).xlsx
+++ b/Mercado Viejo (hay que cambiarlo).xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\Rol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\arkanor-assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42034E8F-1553-4F53-98B8-87DFFA1CCECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8130BBE6-7C05-4C68-90FD-630D032E592B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="821" firstSheet="2" activeTab="2" xr2:uid="{4AA185A2-C228-48BA-9BBC-BFED0B2DEF8B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="821" xr2:uid="{4AA185A2-C228-48BA-9BBC-BFED0B2DEF8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Armas" sheetId="1" r:id="rId1"/>
@@ -2156,7 +2156,7 @@
     <t>Jengibre</t>
   </si>
   <si>
-    <t>solar</t>
+    <t>argentae</t>
   </si>
 </sst>
 </file>
@@ -10249,15 +10249,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>82827</xdr:colOff>
+      <xdr:colOff>14768</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>19915</xdr:rowOff>
+      <xdr:rowOff>19686</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
-      <xdr:colOff>629478</xdr:colOff>
+      <xdr:colOff>742361</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>181978</xdr:rowOff>
+      <xdr:rowOff>361503</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -10286,8 +10286,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="20656827" y="3730524"/>
-          <a:ext cx="546651" cy="537738"/>
+          <a:off x="19064768" y="5353686"/>
+          <a:ext cx="727593" cy="722817"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -10749,15 +10749,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>104776</xdr:colOff>
+      <xdr:colOff>46769</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>19051</xdr:rowOff>
+      <xdr:rowOff>50263</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>657225</xdr:colOff>
+      <xdr:colOff>715232</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>194582</xdr:rowOff>
+      <xdr:rowOff>342665</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -10786,8 +10786,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12296776" y="4924426"/>
-          <a:ext cx="552449" cy="552449"/>
+          <a:off x="11476769" y="6908263"/>
+          <a:ext cx="668463" cy="673402"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -28610,7 +28610,7 @@
         <v>39</v>
       </c>
       <c r="S13" s="172" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="T13" s="105" t="s">
         <v>18</v>
@@ -30938,7 +30938,7 @@
         <v>297</v>
       </c>
       <c r="B1" s="30">
-        <v>3</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -30946,7 +30946,7 @@
         <v>298</v>
       </c>
       <c r="B2" s="32" t="s">
-        <v>362</v>
+        <v>471</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -30954,7 +30954,7 @@
         <v>299</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>471</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B4" s="32">
         <f>B1*INDEX('Tasas de Conversión'!B2:E5,MATCH(B2,'Tasas de Conversión'!A2:A5,0),MATCH(B3,'Tasas de Conversión'!B1:E1,0))</f>
-        <v>6</v>
+        <v>40.800000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>